<commit_message>
Recolor both reports with a soothing palette
- Replace the harsh black + bright-red theme with a calm scheme:
  deep teal-slate (#34515B) bands, soft sage accent (#4F7D6E) for grand
  totals/highlights, warm off-white zebra and soft hairlines
- Applies to both the day-wise and the transposed (brands x days) report
  (shared palette) plus the SUMMARY sheet
- Numbers, totals and layout unchanged
</commit_message>
<xml_diff>
--- a/SEPTEMBER 2026 - ZONE SALES REPORT (BRANDS x DAYS).xlsx
+++ b/SEPTEMBER 2026 - ZONE SALES REPORT (BRANDS x DAYS).xlsx
@@ -51,7 +51,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00EF4444"/>
+      <color rgb="009BC3B6"/>
       <sz val="9"/>
     </font>
     <font>
@@ -69,18 +69,18 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00141414"/>
+      <color rgb="002F3E45"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00141414"/>
+      <color rgb="002F3E45"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00D02128"/>
+      <color rgb="004F7D6E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -90,7 +90,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="005A5A5A"/>
+      <color rgb="005C6B72"/>
       <sz val="10"/>
     </font>
     <font>
@@ -108,36 +108,36 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="005A5A5A"/>
+      <color rgb="005C6B72"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00D02128"/>
+      <color rgb="004F7D6E"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00141414"/>
+      <color rgb="002F3E45"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <i val="1"/>
-      <color rgb="008A8A8A"/>
+      <color rgb="008B969D"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00141414"/>
+      <color rgb="002F3E45"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00D02128"/>
+      <color rgb="004F7D6E"/>
       <sz val="11"/>
     </font>
     <font>
@@ -148,13 +148,13 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00141414"/>
+      <color rgb="002F3E45"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <i val="1"/>
-      <color rgb="008A8A8A"/>
+      <color rgb="008B969D"/>
       <sz val="9.5"/>
     </font>
   </fonts>
@@ -167,17 +167,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A0A0A"/>
+        <fgColor rgb="0034515B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D02128"/>
+        <fgColor rgb="004F7D6E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A1A"/>
+        <fgColor rgb="004A6D76"/>
       </patternFill>
     </fill>
     <fill>
@@ -187,12 +187,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F4F4"/>
+        <fgColor rgb="00EDF2EF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAFAFA"/>
+        <fgColor rgb="00F7F5F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -206,16 +206,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E6E6E6"/>
+        <color rgb="00E7E2D9"/>
       </left>
       <right style="thin">
-        <color rgb="00E6E6E6"/>
+        <color rgb="00E7E2D9"/>
       </right>
       <top style="thin">
-        <color rgb="00E6E6E6"/>
+        <color rgb="00E7E2D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E6E6E6"/>
+        <color rgb="00E7E2D9"/>
       </bottom>
     </border>
   </borders>
@@ -729,7 +729,7 @@
             <rPr>
               <rFont val="Segoe UI"/>
               <b val="1"/>
-              <color rgb="FFEF4444"/>
+              <color rgb="FF9BC3B6"/>
               <sz val="22"/>
             </rPr>
             <t>S</t>
@@ -948,7 +948,7 @@
             <rPr>
               <rFont val="Segoe UI"/>
               <b val="1"/>
-              <color rgb="FFEF4444"/>
+              <color rgb="FF9BC3B6"/>
               <sz val="22"/>
             </rPr>
             <t>A</t>
@@ -1902,7 +1902,7 @@
             <rPr>
               <rFont val="Segoe UI"/>
               <b val="1"/>
-              <color rgb="FFEF4444"/>
+              <color rgb="FF9BC3B6"/>
               <sz val="22"/>
             </rPr>
             <t>C</t>
@@ -2877,7 +2877,7 @@
             <rPr>
               <rFont val="Segoe UI"/>
               <b val="1"/>
-              <color rgb="FFEF4444"/>
+              <color rgb="FF9BC3B6"/>
               <sz val="22"/>
             </rPr>
             <t>B</t>

</xml_diff>